<commit_message>
Remove credential file from branch history
</commit_message>
<xml_diff>
--- a/skill_gaps_2026-08-02.xlsx
+++ b/skill_gaps_2026-08-02.xlsx
@@ -22,64 +22,64 @@
     <t>Jobs Mentioning It</t>
   </si>
   <si>
-    <t>deep learning</t>
-  </si>
-  <si>
-    <t>machine learning</t>
-  </si>
-  <si>
-    <t>natural language processing</t>
-  </si>
-  <si>
-    <t>computer vision</t>
-  </si>
-  <si>
-    <t>devops specific skills like docker, kubernetes, or specific experience with ai-driven automation in a devops context</t>
-  </si>
-  <si>
-    <t>devops specific skills like docker, kubernetes, or specific experience with salesforce devops tools beyond salesforce dx</t>
-  </si>
-  <si>
-    <t>financial services cloud</t>
+    <t>microservices</t>
+  </si>
+  <si>
+    <t>java</t>
+  </si>
+  <si>
+    <t>cloud platforms</t>
+  </si>
+  <si>
+    <t>revenue cloud</t>
+  </si>
+  <si>
+    <t>revenue cloud advanced (rca)</t>
+  </si>
+  <si>
+    <t>quote-to-cash</t>
+  </si>
+  <si>
+    <t>client relationship management</t>
+  </si>
+  <si>
+    <t>customer-success mindset</t>
+  </si>
+  <si>
+    <t>product catalogs</t>
+  </si>
+  <si>
+    <t>workflows</t>
   </si>
   <si>
     <t>triggers</t>
   </si>
   <si>
-    <t>ai/ml</t>
-  </si>
-  <si>
-    <t>drug discovery</t>
-  </si>
-  <si>
-    <t>antimicrobial resistance</t>
-  </si>
-  <si>
-    <t>mlops</t>
-  </si>
-  <si>
-    <t>production ai platform</t>
-  </si>
-  <si>
-    <t>cloud platforms</t>
-  </si>
-  <si>
-    <t>ai engineering</t>
-  </si>
-  <si>
-    <t>python (as a primary language)</t>
-  </si>
-  <si>
-    <t>cloud platforms (other than salesforce)</t>
-  </si>
-  <si>
-    <t>aws</t>
-  </si>
-  <si>
-    <t>amazon bedrock</t>
-  </si>
-  <si>
-    <t>agentic ai</t>
+    <t>platform events</t>
+  </si>
+  <si>
+    <t>production support</t>
+  </si>
+  <si>
+    <t>stakeholder management</t>
+  </si>
+  <si>
+    <t>ci/cd experience specific to salesforce field services</t>
+  </si>
+  <si>
+    <t>hr ai vision</t>
+  </si>
+  <si>
+    <t>hr transformation</t>
+  </si>
+  <si>
+    <t>enterprise-ready solutions</t>
+  </si>
+  <si>
+    <t>agentic experiences</t>
+  </si>
+  <si>
+    <t>predictive insights</t>
   </si>
 </sst>
 </file>
@@ -427,7 +427,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -435,7 +435,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -443,7 +443,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -451,7 +451,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>